<commit_message>
Fix OKR template formula errors: add IFERROR progress formulas and detailed guidance to prevent N/A
</commit_message>
<xml_diff>
--- a/data-room/11-appendix/OKRs Templates.xlsx
+++ b/data-room/11-appendix/OKRs Templates.xlsx
@@ -361,7 +361,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -473,8 +473,9 @@
       <c r="F3" t="n">
         <v>60</v>
       </c>
-      <c r="G3" s="8" t="n">
-        <v>0.5</v>
+      <c r="G3" s="8">
+        <f>IFERROR(IF(C3="Binary",IF(E3=0,0,F3/E3),IF(E3=D3,0,(F3-D3)/(E3-D3))),0)</f>
+        <v/>
       </c>
       <c r="H3" t="n">
         <v>8</v>
@@ -505,8 +506,9 @@
       <c r="F4" s="9" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="G4" s="8" t="n">
-        <v>0.38</v>
+      <c r="G4" s="8">
+        <f>IFERROR(IF(C4="Binary",IF(E4=0,0,F4/E4),IF(E4=D4,0,(F4-D4)/(E4-D4))),0)</f>
+        <v/>
       </c>
       <c r="H4" t="n">
         <v>7</v>
@@ -537,8 +539,9 @@
       <c r="F5" t="n">
         <v>0.9</v>
       </c>
-      <c r="G5" s="8" t="n">
-        <v>0.5</v>
+      <c r="G5" s="8">
+        <f>IFERROR(IF(C5="Binary",IF(E5=0,0,F5/E5),IF(E5=D5,0,(F5-D5)/(E5-D5))),0)</f>
+        <v/>
       </c>
       <c r="H5" t="n">
         <v>7</v>
@@ -569,13 +572,208 @@
       <c r="F6" t="n">
         <v>8</v>
       </c>
-      <c r="G6" s="8" t="n">
-        <v>0.4</v>
+      <c r="G6" s="8">
+        <f>IFERROR(IF(C6="Binary",IF(E6=0,0,F6/E6),IF(E6=D6,0,(F6-D6)/(E6-D6))),0)</f>
+        <v/>
       </c>
       <c r="H6" t="n">
         <v>8</v>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -760,13 +958,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Calculates how close you are to the Target. This is your main tracking metric.</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>#ERROR!</t>
-        </is>
+          <t>Auto-calculates progress. For Metric KRs: (Current-Start)/(Target-Start). For Binary KRs: Current/Target. Wrapped in IFERROR to prevent #DIV/0! and N/A.</t>
+        </is>
+      </c>
+      <c r="D8" s="3">
+        <f>IFERROR(IF(Crow="Binary",IF(Target=0,0,Current/Target),IF(Target=Start,0,(Current-Start)/(Target-Start))),0)</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -876,8 +1073,9 @@
       <c r="F2" s="4" t="n">
         <v>450</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>0.45</v>
+      <c r="G2" s="5">
+        <f>IFERROR(IF(C2="Binary",IF(E2=0,0,F2/E2),IF(E2=D2,0,(F2-D2)/(E2-D2))),0)</f>
+        <v/>
       </c>
       <c r="H2" s="6" t="n">
         <v>45848</v>
@@ -908,8 +1106,9 @@
       <c r="F3" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>0.35</v>
+      <c r="G3" s="5">
+        <f>IFERROR(IF(C3="Binary",IF(E3=0,0,F3/E3),IF(E3=D3,0,(F3-D3)/(E3-D3))),0)</f>
+        <v/>
       </c>
       <c r="H3" s="6" t="n">
         <v>45787</v>
@@ -940,8 +1139,9 @@
       <c r="F4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="n">
-        <v>1</v>
+      <c r="G4" s="5">
+        <f>IFERROR(IF(C4="Binary",IF(E4=0,0,F4/E4),IF(E4=D4,0,(F4-D4)/(E4-D4))),0)</f>
+        <v/>
       </c>
       <c r="H4" s="6" t="n">
         <v>45940</v>
@@ -972,8 +1172,9 @@
       <c r="F5" s="7" t="n">
         <v>0.09375</v>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>0.5</v>
+      <c r="G5" s="5">
+        <f>IFERROR(IF(C5="Binary",IF(E5=0,0,F5/E5),IF(E5=D5,0,(F5-D5)/(E5-D5))),0)</f>
+        <v/>
       </c>
       <c r="H5" s="6" t="n">
         <v>45879</v>

</xml_diff>